<commit_message>
Alteração - documento de visão
</commit_message>
<xml_diff>
--- a/gq-spinoff/6.Gerenciamento de Projeto/gq-spinoff - Checklist Verificacao de Projeto.xlsx
+++ b/gq-spinoff/6.Gerenciamento de Projeto/gq-spinoff - Checklist Verificacao de Projeto.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C78949E-91EA-4999-88E6-FEEB90E73C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC2BDA2-87C4-4913-9276-8E02E25F8233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="6" r:id="rId1"/>
@@ -710,7 +710,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="118">
   <si>
     <t>Ambiente</t>
   </si>
@@ -1070,7 +1070,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1186,6 +1186,14 @@
     <font>
       <b/>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1396,7 +1404,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1465,22 +1473,13 @@
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1489,11 +1488,32 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1504,18 +1524,7 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1851,7 +1860,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.8</c:v>
@@ -1964,7 +1973,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.2</c:v>
@@ -2086,7 +2095,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2199,7 +2208,7 @@
                   <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -7304,17 +7313,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:2" ht="18">
+      <c r="A1" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="41"/>
+      <c r="B1" s="40"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="18" t="s">
@@ -7375,16 +7384,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E6B2C1B-A599-4159-99C1-DE703E343043}">
   <dimension ref="A1:R37"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" customWidth="1"/>
-    <col min="5" max="5" width="6.42578125" customWidth="1"/>
-    <col min="6" max="6" width="6.85546875" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="8.109375" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.88671875" customWidth="1"/>
+    <col min="5" max="5" width="6.44140625" customWidth="1"/>
+    <col min="6" max="6" width="6.88671875" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -7425,11 +7434,11 @@
       </c>
       <c r="B2" s="25">
         <f>('Ver-Iniciação1'!$G$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="25">
         <f>('Ver-Iniciação1'!$H$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="25">
         <f>('Ver-Iniciação1'!$I$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
@@ -7553,11 +7562,11 @@
       </c>
       <c r="D5" s="25">
         <f>('Ver-Iniciação1'!$I$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E5" s="25">
         <f>('Ver-Iniciação1'!$J$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N5" t="s">
         <v>4</v>
@@ -8408,58 +8417,58 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
     <col min="3" max="3" width="84" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.88671875" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="6.140625" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="4.44140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="6.109375" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="6" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="35"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="37"/>
+      <c r="E2" s="39"/>
       <c r="F2" s="21">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>0.73684210526315785</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A3" s="35" t="s">
+    <row r="3" spans="1:10" ht="15" thickBot="1">
+      <c r="A3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="35"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
-    </row>
-    <row r="4" spans="1:10" ht="15">
+      <c r="E3" s="36"/>
+      <c r="F3" s="37"/>
+    </row>
+    <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -8479,8 +8488,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15">
-      <c r="A5" s="28" t="s">
+    <row r="5" spans="1:10" ht="14.4">
+      <c r="A5" s="33" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="9"/>
@@ -8492,11 +8501,11 @@
       <c r="F5" s="12"/>
       <c r="G5">
         <f>COUNTIF(D6,"Sim")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <f>COUNTIF(D6,"Parcialmente")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <f>COUNTIF(D6,"Não")</f>
@@ -8507,22 +8516,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15">
-      <c r="A6" s="33"/>
+    <row r="6" spans="1:10" ht="14.4">
+      <c r="A6" s="34"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>114</v>
+      <c r="D6" s="45" t="s">
+        <v>115</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="9"/>
@@ -8550,7 +8559,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1">
-      <c r="A8" s="29"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="22">
         <v>2</v>
       </c>
@@ -8563,8 +8572,8 @@
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" spans="1:10" ht="15">
-      <c r="A9" s="29"/>
+    <row r="9" spans="1:10" ht="14.4">
+      <c r="A9" s="30"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
@@ -8577,8 +8586,8 @@
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
     </row>
-    <row r="10" spans="1:10" ht="15">
-      <c r="A10" s="29"/>
+    <row r="10" spans="1:10" ht="14.4">
+      <c r="A10" s="30"/>
       <c r="B10" s="5">
         <v>4</v>
       </c>
@@ -8591,8 +8600,8 @@
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
     </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="15">
-      <c r="A11" s="29"/>
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="14.4">
+      <c r="A11" s="30"/>
       <c r="B11" s="5">
         <v>5</v>
       </c>
@@ -8606,7 +8615,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A12" s="29"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="5">
         <v>6</v>
       </c>
@@ -8619,8 +8628,8 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="15">
-      <c r="A13" s="29"/>
+    <row r="13" spans="1:10" ht="14.4">
+      <c r="A13" s="30"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>3</v>
@@ -8645,8 +8654,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="30">
-      <c r="A14" s="29"/>
+    <row r="14" spans="1:10" ht="28.8">
+      <c r="A14" s="30"/>
       <c r="B14" s="23">
         <v>7</v>
       </c>
@@ -8659,8 +8668,8 @@
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A15" s="29"/>
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A15" s="30"/>
       <c r="B15" s="5">
         <v>8</v>
       </c>
@@ -8673,8 +8682,8 @@
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A16" s="29"/>
+    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A16" s="30"/>
       <c r="B16" s="5">
         <v>9</v>
       </c>
@@ -8687,8 +8696,8 @@
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A17" s="29"/>
+    <row r="17" spans="1:10" s="1" customFormat="1" ht="14.4">
+      <c r="A17" s="30"/>
       <c r="B17" s="23">
         <v>10</v>
       </c>
@@ -8701,8 +8710,8 @@
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:10" s="1" customFormat="1" ht="15">
-      <c r="A18" s="29"/>
+    <row r="18" spans="1:10" s="1" customFormat="1" ht="14.4">
+      <c r="A18" s="30"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -8715,8 +8724,8 @@
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" spans="1:10" ht="15">
-      <c r="A19" s="29"/>
+    <row r="19" spans="1:10" ht="14.4">
+      <c r="A19" s="30"/>
       <c r="B19" s="9"/>
       <c r="C19" s="10" t="s">
         <v>97</v>
@@ -8734,15 +8743,15 @@
       </c>
       <c r="I19">
         <f>COUNTIF(D20:D21,"Não")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <f>COUNTIF(D20:D21,"NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="30">
-      <c r="A20" s="29"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="28.8">
+      <c r="A20" s="30"/>
       <c r="B20" s="23">
         <v>12</v>
       </c>
@@ -8755,8 +8764,8 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="30">
-      <c r="A21" s="29"/>
+    <row r="21" spans="1:10" ht="28.8">
+      <c r="A21" s="30"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -8764,13 +8773,13 @@
         <v>80</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="15">
-      <c r="A22" s="29"/>
+    <row r="22" spans="1:10" ht="14.4">
+      <c r="A22" s="30"/>
       <c r="B22" s="9"/>
       <c r="C22" s="10" t="s">
         <v>4</v>
@@ -8795,8 +8804,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="30">
-      <c r="A23" s="29"/>
+    <row r="23" spans="1:10" ht="28.8">
+      <c r="A23" s="30"/>
       <c r="B23" s="23">
         <v>14</v>
       </c>
@@ -8809,8 +8818,8 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:10" ht="15">
-      <c r="A24" s="29"/>
+    <row r="24" spans="1:10" ht="14.4">
+      <c r="A24" s="30"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -8823,8 +8832,8 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="1:10" ht="15">
-      <c r="A25" s="29"/>
+    <row r="25" spans="1:10" ht="14.4">
+      <c r="A25" s="30"/>
       <c r="B25" s="9"/>
       <c r="C25" s="10" t="s">
         <v>36</v>
@@ -8849,8 +8858,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="30">
-      <c r="A26" s="29"/>
+    <row r="26" spans="1:10" ht="28.8">
+      <c r="A26" s="30"/>
       <c r="B26" s="23">
         <v>16</v>
       </c>
@@ -8863,8 +8872,8 @@
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:10" ht="15">
-      <c r="A27" s="29"/>
+    <row r="27" spans="1:10" ht="14.4">
+      <c r="A27" s="30"/>
       <c r="B27" s="5">
         <v>17</v>
       </c>
@@ -8877,8 +8886,8 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="15">
-      <c r="A28" s="29"/>
+    <row r="28" spans="1:10" ht="14.4">
+      <c r="A28" s="30"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>13</v>
@@ -8888,7 +8897,7 @@
       <c r="F28" s="12"/>
       <c r="G28">
         <f>COUNTIF(D29:D36,"Sim")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28">
         <f>COUNTIF(D29:D36,"Parcialmente")</f>
@@ -8903,8 +8912,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="30">
-      <c r="A29" s="29"/>
+    <row r="29" spans="1:10" ht="28.8">
+      <c r="A29" s="30"/>
       <c r="B29" s="23">
         <v>21</v>
       </c>
@@ -8915,8 +8924,8 @@
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
     </row>
-    <row r="30" spans="1:10" ht="15">
-      <c r="A30" s="29"/>
+    <row r="30" spans="1:10" ht="14.4">
+      <c r="A30" s="30"/>
       <c r="B30" s="5">
         <v>22</v>
       </c>
@@ -8929,8 +8938,8 @@
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:10" ht="15">
-      <c r="A31" s="29"/>
+    <row r="31" spans="1:10" ht="14.4">
+      <c r="A31" s="30"/>
       <c r="B31" s="5">
         <v>23</v>
       </c>
@@ -8941,8 +8950,8 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:10" ht="15">
-      <c r="A32" s="29"/>
+    <row r="32" spans="1:10" ht="14.4">
+      <c r="A32" s="30"/>
       <c r="B32" s="5">
         <v>24</v>
       </c>
@@ -8953,8 +8962,8 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="15">
-      <c r="A33" s="29"/>
+    <row r="33" spans="1:10" ht="14.4">
+      <c r="A33" s="30"/>
       <c r="B33" s="5">
         <v>25</v>
       </c>
@@ -8965,8 +8974,8 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="30">
-      <c r="A34" s="29"/>
+    <row r="34" spans="1:10" ht="14.4">
+      <c r="A34" s="30"/>
       <c r="B34" s="5">
         <v>26</v>
       </c>
@@ -8977,19 +8986,21 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A35" s="29"/>
+      <c r="A35" s="30"/>
       <c r="B35" s="5">
         <v>27</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="3"/>
+      <c r="D35" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="E35" s="8"/>
       <c r="F35" s="8"/>
     </row>
-    <row r="36" spans="1:10" ht="15">
-      <c r="A36" s="29"/>
+    <row r="36" spans="1:10" ht="14.4">
+      <c r="A36" s="30"/>
       <c r="B36" s="5">
         <v>28</v>
       </c>
@@ -9001,7 +9012,7 @@
       <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1">
-      <c r="A37" s="31" t="s">
+      <c r="A37" s="28" t="s">
         <v>30</v>
       </c>
       <c r="B37" s="9"/>
@@ -9028,8 +9039,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="30">
-      <c r="A38" s="32"/>
+    <row r="38" spans="1:10" ht="28.8">
+      <c r="A38" s="29"/>
       <c r="B38" s="23">
         <v>30</v>
       </c>
@@ -9042,8 +9053,8 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="30">
-      <c r="A39" s="32"/>
+    <row r="39" spans="1:10" ht="14.4">
+      <c r="A39" s="29"/>
       <c r="B39" s="5">
         <v>31</v>
       </c>
@@ -9054,8 +9065,8 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:10" ht="15">
-      <c r="A40" s="32"/>
+    <row r="40" spans="1:10" ht="14.4">
+      <c r="A40" s="29"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
@@ -9069,7 +9080,7 @@
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="20.25" customHeight="1">
-      <c r="A41" s="32"/>
+      <c r="A41" s="29"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -9106,55 +9117,55 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
     <col min="3" max="3" width="68" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
     <col min="7" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="35"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="37"/>
+      <c r="E2" s="39"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D42)-COUNTIF(D5:D42,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A3" s="35" t="s">
+    <row r="3" spans="1:10" ht="15" thickBot="1">
+      <c r="A3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="35"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="39"/>
-      <c r="F3" s="40"/>
-    </row>
-    <row r="4" spans="1:10" ht="15">
+      <c r="E3" s="43"/>
+      <c r="F3" s="44"/>
+    </row>
+    <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -9175,7 +9186,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9186,8 +9197,8 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="15">
-      <c r="A6" s="29"/>
+    <row r="6" spans="1:10" ht="14.4">
+      <c r="A6" s="30"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -9214,8 +9225,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15">
-      <c r="A7" s="29"/>
+    <row r="7" spans="1:10" ht="14.4">
+      <c r="A7" s="30"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9224,8 +9235,8 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A8" s="29"/>
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A8" s="30"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -9252,8 +9263,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A9" s="29"/>
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A9" s="30"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
@@ -9268,8 +9279,8 @@
       <c r="I9"/>
       <c r="J9"/>
     </row>
-    <row r="10" spans="1:10" ht="15">
-      <c r="A10" s="29"/>
+    <row r="10" spans="1:10" ht="14.4">
+      <c r="A10" s="30"/>
       <c r="B10" s="9"/>
       <c r="C10" s="10" t="s">
         <v>97</v>
@@ -9278,8 +9289,8 @@
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="30">
-      <c r="A11" s="29"/>
+    <row r="11" spans="1:10" ht="28.8">
+      <c r="A11" s="30"/>
       <c r="B11" s="23">
         <v>4</v>
       </c>
@@ -9306,8 +9317,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30">
-      <c r="A12" s="29"/>
+    <row r="12" spans="1:10" ht="28.8">
+      <c r="A12" s="30"/>
       <c r="B12" s="23">
         <v>5</v>
       </c>
@@ -9318,8 +9329,8 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="30">
-      <c r="A13" s="29"/>
+    <row r="13" spans="1:10" ht="14.4">
+      <c r="A13" s="30"/>
       <c r="B13" s="5">
         <v>6</v>
       </c>
@@ -9330,8 +9341,8 @@
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="30">
-      <c r="A14" s="29"/>
+    <row r="14" spans="1:10" ht="28.8">
+      <c r="A14" s="30"/>
       <c r="B14" s="5">
         <v>7</v>
       </c>
@@ -9342,8 +9353,8 @@
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="15">
-      <c r="A15" s="29"/>
+    <row r="15" spans="1:10" ht="14.4">
+      <c r="A15" s="30"/>
       <c r="B15" s="9"/>
       <c r="C15" s="10" t="s">
         <v>4</v>
@@ -9352,8 +9363,8 @@
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="15">
-      <c r="A16" s="29"/>
+    <row r="16" spans="1:10" ht="14.4">
+      <c r="A16" s="30"/>
       <c r="B16" s="5">
         <v>7</v>
       </c>
@@ -9381,7 +9392,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="9"/>
@@ -9392,8 +9403,8 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="30">
-      <c r="A18" s="29"/>
+    <row r="18" spans="1:10" ht="28.8">
+      <c r="A18" s="30"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
@@ -9420,8 +9431,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="30">
-      <c r="A19" s="29"/>
+    <row r="19" spans="1:10" ht="28.8">
+      <c r="A19" s="30"/>
       <c r="B19" s="23">
         <v>10</v>
       </c>
@@ -9432,8 +9443,8 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A20" s="29"/>
+    <row r="20" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A20" s="30"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
@@ -9444,8 +9455,8 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="45">
-      <c r="A21" s="29"/>
+    <row r="21" spans="1:10" ht="28.8">
+      <c r="A21" s="30"/>
       <c r="B21" s="5">
         <v>12</v>
       </c>
@@ -9456,8 +9467,8 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="15">
-      <c r="A22" s="28" t="s">
+    <row r="22" spans="1:10" ht="14.4">
+      <c r="A22" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="9"/>
@@ -9468,8 +9479,8 @@
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="30">
-      <c r="A23" s="29"/>
+    <row r="23" spans="1:10" ht="28.8">
+      <c r="A23" s="30"/>
       <c r="B23" s="5">
         <v>17</v>
       </c>
@@ -9496,8 +9507,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="30">
-      <c r="A24" s="29"/>
+    <row r="24" spans="1:10" ht="28.8">
+      <c r="A24" s="30"/>
       <c r="B24" s="5">
         <v>18</v>
       </c>
@@ -9508,8 +9519,8 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="1:10" ht="30">
-      <c r="A25" s="29"/>
+    <row r="25" spans="1:10" ht="28.8">
+      <c r="A25" s="30"/>
       <c r="B25" s="5">
         <v>19</v>
       </c>
@@ -9520,8 +9531,8 @@
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:10" ht="15">
-      <c r="A26" s="29"/>
+    <row r="26" spans="1:10" ht="14.4">
+      <c r="A26" s="30"/>
       <c r="B26" s="5">
         <v>21</v>
       </c>
@@ -9532,8 +9543,8 @@
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:10" ht="15">
-      <c r="A27" s="29"/>
+    <row r="27" spans="1:10" ht="14.4">
+      <c r="A27" s="30"/>
       <c r="B27" s="5">
         <v>22</v>
       </c>
@@ -9544,8 +9555,8 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="15">
-      <c r="A28" s="30" t="s">
+    <row r="28" spans="1:10" ht="14.4">
+      <c r="A28" s="41" t="s">
         <v>11</v>
       </c>
       <c r="B28" s="9"/>
@@ -9556,8 +9567,8 @@
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
     </row>
-    <row r="29" spans="1:10" ht="15">
-      <c r="A29" s="30"/>
+    <row r="29" spans="1:10" ht="14.4">
+      <c r="A29" s="41"/>
       <c r="B29" s="5">
         <v>23</v>
       </c>
@@ -9584,8 +9595,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15">
-      <c r="A30" s="30"/>
+    <row r="30" spans="1:10" ht="14.4">
+      <c r="A30" s="41"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
@@ -9596,8 +9607,8 @@
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:10" ht="30">
-      <c r="A31" s="30"/>
+    <row r="31" spans="1:10" ht="28.8">
+      <c r="A31" s="41"/>
       <c r="B31" s="5">
         <v>25</v>
       </c>
@@ -9608,8 +9619,8 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:10" ht="15">
-      <c r="A32" s="30"/>
+    <row r="32" spans="1:10" ht="14.4">
+      <c r="A32" s="41"/>
       <c r="B32" s="5">
         <v>26</v>
       </c>
@@ -9620,8 +9631,8 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="15">
-      <c r="A33" s="30"/>
+    <row r="33" spans="1:10" ht="14.4">
+      <c r="A33" s="41"/>
       <c r="B33" s="5">
         <v>27</v>
       </c>
@@ -9632,8 +9643,8 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="15">
-      <c r="A34" s="30"/>
+    <row r="34" spans="1:10" ht="14.4">
+      <c r="A34" s="41"/>
       <c r="B34" s="5">
         <v>28</v>
       </c>
@@ -9645,7 +9656,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="31" t="s">
+      <c r="A35" s="28" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -9656,8 +9667,8 @@
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
     </row>
-    <row r="36" spans="1:10" ht="30">
-      <c r="A36" s="32"/>
+    <row r="36" spans="1:10" ht="28.8">
+      <c r="A36" s="29"/>
       <c r="B36" s="5">
         <v>29</v>
       </c>
@@ -9684,8 +9695,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="15">
-      <c r="A37" s="32"/>
+    <row r="37" spans="1:10" ht="14.4">
+      <c r="A37" s="29"/>
       <c r="B37" s="5">
         <v>30</v>
       </c>
@@ -9696,8 +9707,8 @@
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:10" ht="30">
-      <c r="A38" s="32"/>
+    <row r="38" spans="1:10" ht="28.8">
+      <c r="A38" s="29"/>
       <c r="B38" s="5">
         <v>31</v>
       </c>
@@ -9708,8 +9719,8 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="15">
-      <c r="A39" s="32"/>
+    <row r="39" spans="1:10" ht="14.4">
+      <c r="A39" s="29"/>
       <c r="B39" s="9"/>
       <c r="C39" s="10" t="s">
         <v>15</v>
@@ -9718,8 +9729,8 @@
       <c r="E39" s="12"/>
       <c r="F39" s="12"/>
     </row>
-    <row r="40" spans="1:10" ht="15">
-      <c r="A40" s="32"/>
+    <row r="40" spans="1:10" ht="14.4">
+      <c r="A40" s="29"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
@@ -9746,8 +9757,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="15">
-      <c r="A41" s="32"/>
+    <row r="41" spans="1:10" ht="14.4">
+      <c r="A41" s="29"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -9787,55 +9798,55 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J57"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="71.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
-    <col min="7" max="10" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="71.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="7" max="10" width="9.109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="35"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="37"/>
+      <c r="E2" s="39"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D42,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A3" s="35" t="s">
+    <row r="3" spans="1:10" ht="15" thickBot="1">
+      <c r="A3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="35"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="39"/>
-      <c r="F3" s="40"/>
-    </row>
-    <row r="4" spans="1:10" ht="15">
+      <c r="E3" s="43"/>
+      <c r="F3" s="44"/>
+    </row>
+    <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -9856,7 +9867,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9867,8 +9878,8 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="15">
-      <c r="A6" s="29"/>
+    <row r="6" spans="1:10" ht="14.4">
+      <c r="A6" s="30"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -9895,8 +9906,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15">
-      <c r="A7" s="29"/>
+    <row r="7" spans="1:10" ht="14.4">
+      <c r="A7" s="30"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9905,8 +9916,8 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A8" s="29"/>
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A8" s="30"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -9933,8 +9944,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15">
-      <c r="A9" s="29"/>
+    <row r="9" spans="1:10" ht="14.4">
+      <c r="A9" s="30"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>97</v>
@@ -9943,8 +9954,8 @@
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="30">
-      <c r="A10" s="29"/>
+    <row r="10" spans="1:10" ht="28.8">
+      <c r="A10" s="30"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -9971,8 +9982,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30">
-      <c r="A11" s="29"/>
+    <row r="11" spans="1:10" ht="28.8">
+      <c r="A11" s="30"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -9984,7 +9995,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A12" s="29"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -9995,8 +10006,8 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="15">
-      <c r="A13" s="29"/>
+    <row r="13" spans="1:10" ht="14.4">
+      <c r="A13" s="30"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10005,8 +10016,8 @@
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
     </row>
-    <row r="14" spans="1:10" ht="15">
-      <c r="A14" s="29"/>
+    <row r="14" spans="1:10" ht="14.4">
+      <c r="A14" s="30"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10034,7 +10045,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10045,8 +10056,8 @@
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="15">
-      <c r="A16" s="29"/>
+    <row r="16" spans="1:10" ht="14.4">
+      <c r="A16" s="30"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10073,8 +10084,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15">
-      <c r="A17" s="28" t="s">
+    <row r="17" spans="1:10" ht="14.4">
+      <c r="A17" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10085,8 +10096,8 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="15">
-      <c r="A18" s="29"/>
+    <row r="18" spans="1:10" ht="14.4">
+      <c r="A18" s="30"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -10113,8 +10124,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="30">
-      <c r="A19" s="29"/>
+    <row r="19" spans="1:10" ht="28.8">
+      <c r="A19" s="30"/>
       <c r="B19" s="5">
         <v>13</v>
       </c>
@@ -10125,8 +10136,8 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:10" ht="30">
-      <c r="A20" s="29"/>
+    <row r="20" spans="1:10" ht="28.8">
+      <c r="A20" s="30"/>
       <c r="B20" s="5">
         <v>14</v>
       </c>
@@ -10137,8 +10148,8 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="15">
-      <c r="A21" s="29"/>
+    <row r="21" spans="1:10" ht="14.4">
+      <c r="A21" s="30"/>
       <c r="B21" s="5">
         <v>15</v>
       </c>
@@ -10149,8 +10160,8 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="15">
-      <c r="A22" s="29"/>
+    <row r="22" spans="1:10" ht="14.4">
+      <c r="A22" s="30"/>
       <c r="B22" s="5">
         <v>16</v>
       </c>
@@ -10161,8 +10172,8 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="1:10" ht="15">
-      <c r="A23" s="28" t="s">
+    <row r="23" spans="1:10" ht="14.4">
+      <c r="A23" s="33" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="9"/>
@@ -10173,8 +10184,8 @@
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" spans="1:10" ht="30">
-      <c r="A24" s="29"/>
+    <row r="24" spans="1:10" ht="28.8">
+      <c r="A24" s="30"/>
       <c r="B24" s="23">
         <v>17</v>
       </c>
@@ -10201,8 +10212,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="30">
-      <c r="A25" s="29"/>
+    <row r="25" spans="1:10" ht="28.8">
+      <c r="A25" s="30"/>
       <c r="B25" s="5">
         <v>18</v>
       </c>
@@ -10213,8 +10224,8 @@
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:10" ht="15">
-      <c r="A26" s="29"/>
+    <row r="26" spans="1:10" ht="14.4">
+      <c r="A26" s="30"/>
       <c r="B26" s="5">
         <v>19</v>
       </c>
@@ -10225,8 +10236,8 @@
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:10" ht="15">
-      <c r="A27" s="29"/>
+    <row r="27" spans="1:10" ht="14.4">
+      <c r="A27" s="30"/>
       <c r="B27" s="5">
         <v>21</v>
       </c>
@@ -10237,8 +10248,8 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="15">
-      <c r="A28" s="29"/>
+    <row r="28" spans="1:10" ht="14.4">
+      <c r="A28" s="30"/>
       <c r="B28" s="5">
         <v>22</v>
       </c>
@@ -10249,8 +10260,8 @@
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="1:10" ht="15">
-      <c r="A29" s="30" t="s">
+    <row r="29" spans="1:10" ht="14.4">
+      <c r="A29" s="41" t="s">
         <v>11</v>
       </c>
       <c r="B29" s="9"/>
@@ -10261,8 +10272,8 @@
       <c r="E29" s="12"/>
       <c r="F29" s="12"/>
     </row>
-    <row r="30" spans="1:10" ht="15">
-      <c r="A30" s="30"/>
+    <row r="30" spans="1:10" ht="14.4">
+      <c r="A30" s="41"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
@@ -10289,8 +10300,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="30">
-      <c r="A31" s="30"/>
+    <row r="31" spans="1:10" ht="28.8">
+      <c r="A31" s="41"/>
       <c r="B31" s="5">
         <v>26</v>
       </c>
@@ -10301,8 +10312,8 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:10" ht="15">
-      <c r="A32" s="30"/>
+    <row r="32" spans="1:10" ht="14.4">
+      <c r="A32" s="41"/>
       <c r="B32" s="5">
         <v>27</v>
       </c>
@@ -10313,8 +10324,8 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="15">
-      <c r="A33" s="30"/>
+    <row r="33" spans="1:10" ht="14.4">
+      <c r="A33" s="41"/>
       <c r="B33" s="5">
         <v>28</v>
       </c>
@@ -10325,8 +10336,8 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="15">
-      <c r="A34" s="30"/>
+    <row r="34" spans="1:10" ht="14.4">
+      <c r="A34" s="41"/>
       <c r="B34" s="5">
         <v>29</v>
       </c>
@@ -10338,7 +10349,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="31" t="s">
+      <c r="A35" s="28" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -10349,8 +10360,8 @@
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
     </row>
-    <row r="36" spans="1:10" ht="30">
-      <c r="A36" s="32"/>
+    <row r="36" spans="1:10" ht="28.8">
+      <c r="A36" s="29"/>
       <c r="B36" s="5">
         <v>30</v>
       </c>
@@ -10377,8 +10388,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="15">
-      <c r="A37" s="32"/>
+    <row r="37" spans="1:10" ht="14.4">
+      <c r="A37" s="29"/>
       <c r="B37" s="5">
         <v>31</v>
       </c>
@@ -10389,8 +10400,8 @@
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:10" ht="30">
-      <c r="A38" s="32"/>
+    <row r="38" spans="1:10" ht="28.8">
+      <c r="A38" s="29"/>
       <c r="B38" s="5">
         <v>32</v>
       </c>
@@ -10401,8 +10412,8 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="15">
-      <c r="A39" s="32"/>
+    <row r="39" spans="1:10" ht="14.4">
+      <c r="A39" s="29"/>
       <c r="B39" s="5"/>
       <c r="C39" s="8" t="s">
         <v>105</v>
@@ -10411,8 +10422,8 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:10" ht="15">
-      <c r="A40" s="32"/>
+    <row r="40" spans="1:10" ht="14.4">
+      <c r="A40" s="29"/>
       <c r="B40" s="9"/>
       <c r="C40" s="10" t="s">
         <v>15</v>
@@ -10421,8 +10432,8 @@
       <c r="E40" s="12"/>
       <c r="F40" s="12"/>
     </row>
-    <row r="41" spans="1:10" ht="15">
-      <c r="A41" s="32"/>
+    <row r="41" spans="1:10" ht="14.4">
+      <c r="A41" s="29"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -10449,8 +10460,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="15">
-      <c r="A42" s="32"/>
+    <row r="42" spans="1:10" ht="14.4">
+      <c r="A42" s="29"/>
       <c r="B42" s="5">
         <v>34</v>
       </c>
@@ -10461,47 +10472,47 @@
       <c r="E42" s="8"/>
       <c r="F42" s="8"/>
     </row>
-    <row r="51" spans="2:3" ht="15">
+    <row r="51" spans="2:3" ht="14.4">
       <c r="B51"/>
       <c r="C51"/>
     </row>
-    <row r="52" spans="2:3" ht="15">
+    <row r="52" spans="2:3" ht="14.4">
       <c r="B52"/>
       <c r="C52"/>
     </row>
-    <row r="53" spans="2:3" ht="15">
+    <row r="53" spans="2:3" ht="14.4">
       <c r="B53"/>
       <c r="C53"/>
     </row>
-    <row r="54" spans="2:3" ht="15">
+    <row r="54" spans="2:3" ht="14.4">
       <c r="B54"/>
       <c r="C54"/>
     </row>
-    <row r="55" spans="2:3" ht="15">
+    <row r="55" spans="2:3" ht="14.4">
       <c r="B55"/>
       <c r="C55"/>
     </row>
-    <row r="56" spans="2:3" ht="15">
+    <row r="56" spans="2:3" ht="14.4">
       <c r="B56"/>
       <c r="C56"/>
     </row>
-    <row r="57" spans="2:3" ht="15">
+    <row r="57" spans="2:3" ht="14.4">
       <c r="B57"/>
       <c r="C57"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:F3"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A17:A22"/>
     <mergeCell ref="A29:A34"/>
     <mergeCell ref="A35:A42"/>
     <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23 D15 D17 D40 D35 D29" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -10519,55 +10530,55 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J58"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="71.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="71.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
     <col min="7" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="35"/>
+      <c r="B2" s="32"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="37"/>
+      <c r="E2" s="39"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D43,"Sim")/(COUNTA(D5:D43)-COUNTIF(D5:D43,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A3" s="35" t="s">
+    <row r="3" spans="1:10" ht="15" thickBot="1">
+      <c r="A3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="35"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="38" t="s">
+      <c r="D3" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="39"/>
-      <c r="F3" s="40"/>
-    </row>
-    <row r="4" spans="1:10" ht="15">
+      <c r="E3" s="43"/>
+      <c r="F3" s="44"/>
+    </row>
+    <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -10588,7 +10599,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -10599,8 +10610,8 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="15">
-      <c r="A6" s="29"/>
+    <row r="6" spans="1:10" ht="14.4">
+      <c r="A6" s="30"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -10627,8 +10638,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15">
-      <c r="A7" s="29"/>
+    <row r="7" spans="1:10" ht="14.4">
+      <c r="A7" s="30"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -10637,8 +10648,8 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A8" s="29"/>
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A8" s="30"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -10665,8 +10676,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15">
-      <c r="A9" s="29"/>
+    <row r="9" spans="1:10" ht="14.4">
+      <c r="A9" s="30"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>14</v>
@@ -10675,8 +10686,8 @@
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="30">
-      <c r="A10" s="29"/>
+    <row r="10" spans="1:10" ht="28.8">
+      <c r="A10" s="30"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -10703,8 +10714,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30">
-      <c r="A11" s="29"/>
+    <row r="11" spans="1:10" ht="28.8">
+      <c r="A11" s="30"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -10716,7 +10727,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="29.25" customHeight="1">
-      <c r="A12" s="29"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -10727,8 +10738,8 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="15">
-      <c r="A13" s="29"/>
+    <row r="13" spans="1:10" ht="14.4">
+      <c r="A13" s="30"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10737,8 +10748,8 @@
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
     </row>
-    <row r="14" spans="1:10" ht="15">
-      <c r="A14" s="29"/>
+    <row r="14" spans="1:10" ht="14.4">
+      <c r="A14" s="30"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10766,7 +10777,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10777,8 +10788,8 @@
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="15">
-      <c r="A16" s="29"/>
+    <row r="16" spans="1:10" ht="14.4">
+      <c r="A16" s="30"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10806,7 +10817,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10817,8 +10828,8 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="30">
-      <c r="A18" s="29"/>
+    <row r="18" spans="1:10" ht="14.4">
+      <c r="A18" s="30"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
@@ -10845,8 +10856,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15">
-      <c r="A19" s="29"/>
+    <row r="19" spans="1:10" ht="14.4">
+      <c r="A19" s="30"/>
       <c r="B19" s="5">
         <v>10</v>
       </c>
@@ -10857,8 +10868,8 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:10" ht="30">
-      <c r="A20" s="29"/>
+    <row r="20" spans="1:10" ht="28.8">
+      <c r="A20" s="30"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
@@ -10869,8 +10880,8 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="15">
-      <c r="A21" s="33"/>
+    <row r="21" spans="1:10" ht="14.4">
+      <c r="A21" s="34"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -10881,8 +10892,8 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="15">
-      <c r="A22" s="28" t="s">
+    <row r="22" spans="1:10" ht="14.4">
+      <c r="A22" s="33" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="9"/>
@@ -10893,8 +10904,8 @@
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="15">
-      <c r="A23" s="29"/>
+    <row r="23" spans="1:10" ht="14.4">
+      <c r="A23" s="30"/>
       <c r="B23" s="5">
         <v>14</v>
       </c>
@@ -10921,8 +10932,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="15">
-      <c r="A24" s="29"/>
+    <row r="24" spans="1:10" ht="14.4">
+      <c r="A24" s="30"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -10934,7 +10945,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="33" t="s">
         <v>21</v>
       </c>
       <c r="B25" s="9"/>
@@ -10945,8 +10956,8 @@
       <c r="E25" s="12"/>
       <c r="F25" s="12"/>
     </row>
-    <row r="26" spans="1:10" s="1" customFormat="1" ht="30">
-      <c r="A26" s="29"/>
+    <row r="26" spans="1:10" s="1" customFormat="1" ht="28.8">
+      <c r="A26" s="30"/>
       <c r="B26" s="23">
         <v>24</v>
       </c>
@@ -10973,8 +10984,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:10" s="1" customFormat="1" ht="45">
-      <c r="A27" s="29"/>
+    <row r="27" spans="1:10" s="1" customFormat="1" ht="43.2">
+      <c r="A27" s="30"/>
       <c r="B27" s="5">
         <v>25</v>
       </c>
@@ -10985,8 +10996,8 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="15">
-      <c r="A28" s="29"/>
+    <row r="28" spans="1:10" ht="14.4">
+      <c r="A28" s="30"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>10</v>
@@ -10995,8 +11006,8 @@
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
     </row>
-    <row r="29" spans="1:10" ht="30">
-      <c r="A29" s="29"/>
+    <row r="29" spans="1:10" ht="28.8">
+      <c r="A29" s="30"/>
       <c r="B29" s="23">
         <v>26</v>
       </c>
@@ -11023,8 +11034,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15">
-      <c r="A30" s="30" t="s">
+    <row r="30" spans="1:10" ht="14.4">
+      <c r="A30" s="41" t="s">
         <v>11</v>
       </c>
       <c r="B30" s="9"/>
@@ -11035,8 +11046,8 @@
       <c r="E30" s="12"/>
       <c r="F30" s="12"/>
     </row>
-    <row r="31" spans="1:10" ht="15">
-      <c r="A31" s="30"/>
+    <row r="31" spans="1:10" ht="14.4">
+      <c r="A31" s="41"/>
       <c r="B31" s="5">
         <v>19</v>
       </c>
@@ -11063,8 +11074,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="30">
-      <c r="A32" s="30"/>
+    <row r="32" spans="1:10" ht="28.8">
+      <c r="A32" s="41"/>
       <c r="B32" s="5">
         <v>20</v>
       </c>
@@ -11075,8 +11086,8 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="15">
-      <c r="A33" s="30"/>
+    <row r="33" spans="1:10" ht="14.4">
+      <c r="A33" s="41"/>
       <c r="B33" s="5">
         <v>21</v>
       </c>
@@ -11087,8 +11098,8 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="15">
-      <c r="A34" s="30"/>
+    <row r="34" spans="1:10" ht="14.4">
+      <c r="A34" s="41"/>
       <c r="B34" s="5">
         <v>24</v>
       </c>
@@ -11099,8 +11110,8 @@
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" spans="1:10" ht="15">
-      <c r="A35" s="30"/>
+    <row r="35" spans="1:10" ht="14.4">
+      <c r="A35" s="41"/>
       <c r="B35" s="5">
         <v>25</v>
       </c>
@@ -11112,7 +11123,7 @@
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="28" t="s">
         <v>30</v>
       </c>
       <c r="B36" s="9"/>
@@ -11123,8 +11134,8 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="37" spans="1:10" ht="30">
-      <c r="A37" s="32"/>
+    <row r="37" spans="1:10" ht="28.8">
+      <c r="A37" s="29"/>
       <c r="B37" s="5">
         <v>26</v>
       </c>
@@ -11151,8 +11162,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="15">
-      <c r="A38" s="32"/>
+    <row r="38" spans="1:10" ht="14.4">
+      <c r="A38" s="29"/>
       <c r="B38" s="5">
         <v>27</v>
       </c>
@@ -11163,8 +11174,8 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="30">
-      <c r="A39" s="32"/>
+    <row r="39" spans="1:10" ht="28.8">
+      <c r="A39" s="29"/>
       <c r="B39" s="5">
         <v>28</v>
       </c>
@@ -11175,8 +11186,8 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:10" ht="15">
-      <c r="A40" s="32"/>
+    <row r="40" spans="1:10" ht="14.4">
+      <c r="A40" s="29"/>
       <c r="B40" s="5"/>
       <c r="C40" s="8" t="s">
         <v>105</v>
@@ -11185,8 +11196,8 @@
       <c r="E40" s="8"/>
       <c r="F40" s="8"/>
     </row>
-    <row r="41" spans="1:10" ht="15">
-      <c r="A41" s="32"/>
+    <row r="41" spans="1:10" ht="14.4">
+      <c r="A41" s="29"/>
       <c r="B41" s="9"/>
       <c r="C41" s="10" t="s">
         <v>15</v>
@@ -11195,8 +11206,8 @@
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
     </row>
-    <row r="42" spans="1:10" ht="15">
-      <c r="A42" s="32"/>
+    <row r="42" spans="1:10" ht="14.4">
+      <c r="A42" s="29"/>
       <c r="B42" s="5">
         <v>29</v>
       </c>
@@ -11223,8 +11234,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="15">
-      <c r="A43" s="32"/>
+    <row r="43" spans="1:10" ht="14.4">
+      <c r="A43" s="29"/>
       <c r="B43" s="5">
         <v>30</v>
       </c>
@@ -11235,36 +11246,41 @@
       <c r="E43" s="8"/>
       <c r="F43" s="8"/>
     </row>
-    <row r="52" spans="2:3" ht="15">
+    <row r="52" spans="2:3" ht="14.4">
       <c r="B52"/>
       <c r="C52"/>
     </row>
-    <row r="53" spans="2:3" ht="15">
+    <row r="53" spans="2:3" ht="14.4">
       <c r="B53"/>
       <c r="C53"/>
     </row>
-    <row r="54" spans="2:3" ht="15">
+    <row r="54" spans="2:3" ht="14.4">
       <c r="B54"/>
       <c r="C54"/>
     </row>
-    <row r="55" spans="2:3" ht="15">
+    <row r="55" spans="2:3" ht="14.4">
       <c r="B55"/>
       <c r="C55"/>
     </row>
-    <row r="56" spans="2:3" ht="15">
+    <row r="56" spans="2:3" ht="14.4">
       <c r="B56"/>
       <c r="C56"/>
     </row>
-    <row r="57" spans="2:3" ht="15">
+    <row r="57" spans="2:3" ht="14.4">
       <c r="B57"/>
       <c r="C57"/>
     </row>
-    <row r="58" spans="2:3" ht="15">
+    <row r="58" spans="2:3" ht="14.4">
       <c r="B58"/>
       <c r="C58"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A25:A29"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:F1"/>
@@ -11272,11 +11288,6 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A25:A29"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D25 D17 D15 D22 D41 D36 D30 D28" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>